<commit_message>
#3 (Alternate Part Added)
</commit_message>
<xml_diff>
--- a/Design Files/LLR-05U (Advance Version)/Secondary Board/BOM/Client BOM LLR-05U (Secondary-Board).xlsx
+++ b/Design Files/LLR-05U (Advance Version)/Secondary Board/BOM/Client BOM LLR-05U (Secondary-Board).xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Secondary Board\Client BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Secondary Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBA88B6-0C96-4240-BEEE-699B92FCA4BC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E31981D-9490-4B7B-944D-F4E69B9326D4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="99">
   <si>
     <t>#</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Alternate Link: https://www.aliexpress.us/item/3256803267239198.html?spm=a2g0o.store_pc_promotion.promoteRecommendProducts_11763439.1005003453553950&amp;gatewayAdapt=glo2usa4itemAdapt</t>
   </si>
 </sst>
 </file>
@@ -818,7 +821,7 @@
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -959,7 +962,7 @@
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="84.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -989,7 +992,9 @@
       <c r="J6" s="9">
         <v>1</v>
       </c>
-      <c r="K6" s="9"/>
+      <c r="K6" s="9" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>

</xml_diff>

<commit_message>
#4 Changes done in SCH and  PCB and Fresh Deliverables generated
</commit_message>
<xml_diff>
--- a/Design Files/LLR-05U (Advance Version)/Secondary Board/BOM/Client BOM LLR-05U (Secondary-Board).xlsx
+++ b/Design Files/LLR-05U (Advance Version)/Secondary Board/BOM/Client BOM LLR-05U (Secondary-Board).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20410"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20411"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Secondary Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Secondary Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E31981D-9490-4B7B-944D-F4E69B9326D4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF2B54B-CF38-492C-969C-8DFDF46970B3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="110">
   <si>
     <t>#</t>
   </si>
@@ -317,6 +317,39 @@
   </si>
   <si>
     <t>Alternate Link: https://www.aliexpress.us/item/3256803267239198.html?spm=a2g0o.store_pc_promotion.promoteRecommendProducts_11763439.1005003453553950&amp;gatewayAdapt=glo2usa4itemAdapt</t>
+  </si>
+  <si>
+    <t>C1, C4, C5, C10, C11, C12</t>
+  </si>
+  <si>
+    <t>CAP CER 10000PF 25V X7R 0402</t>
+  </si>
+  <si>
+    <t>Cap-0402</t>
+  </si>
+  <si>
+    <t>CC0402KRX7R8BB103</t>
+  </si>
+  <si>
+    <t>10nF</t>
+  </si>
+  <si>
+    <t>D1, D2</t>
+  </si>
+  <si>
+    <t>DFN1006-2(0402) ESD Protection Devices ROHS</t>
+  </si>
+  <si>
+    <t>DFN1006-2L (Bi-Directional)</t>
+  </si>
+  <si>
+    <t>ESD5451N</t>
+  </si>
+  <si>
+    <t>TECH PUBLIC</t>
+  </si>
+  <si>
+    <t>Diode</t>
   </si>
 </sst>
 </file>
@@ -809,7 +842,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -870,7 +903,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -880,121 +913,119 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>47</v>
+        <v>102</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="J3" s="7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B18" si="0">ROW(B4) - ROW($B$2)</f>
+        <f>ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I4" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="J4" s="9">
-        <v>2</v>
-      </c>
-      <c r="K4" s="9"/>
+      <c r="D4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="J4" s="7">
+        <v>1</v>
+      </c>
+      <c r="K4" s="7"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
-        <f>ROW(B5) - ROW($B$2)</f>
+        <f t="shared" ref="B5:B20" si="0">ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="7" t="s">
+      <c r="D5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="8"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="J5" s="7">
-        <v>3</v>
-      </c>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="1:11" ht="84.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G5" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="J5" s="9">
+        <v>2</v>
+      </c>
+      <c r="K5" s="9"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B6) - ROW($B$2)</f>
         <v>4</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="J6" s="7">
         <v>3</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="G6" s="10">
-        <v>610010243021</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="J6" s="9">
-        <v>1</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>98</v>
-      </c>
+      <c r="K6" s="7"/>
     </row>
     <row r="7" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
@@ -1003,62 +1034,64 @@
         <v>5</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>4</v>
+        <v>109</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>15</v>
+        <v>104</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>49</v>
+        <v>106</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>58</v>
+        <v>107</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="J7" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="84.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>59</v>
+        <v>96</v>
+      </c>
+      <c r="G8" s="10">
+        <v>610010243021</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I8" s="10" t="s">
         <v>97</v>
       </c>
       <c r="J8" s="9">
-        <v>3</v>
-      </c>
-      <c r="K8" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1067,54 +1100,54 @@
         <v>7</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>97</v>
       </c>
       <c r="J9" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="I10" s="10" t="s">
         <v>97</v>
@@ -1124,99 +1157,99 @@
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
         <v>9</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>97</v>
       </c>
       <c r="J11" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="J12" s="9">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="J13" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K13" s="7"/>
     </row>
@@ -1230,29 +1263,29 @@
         <v>7</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>52</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>79</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J14" s="9">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1262,25 +1295,25 @@
         <v>7</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>52</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J15" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K15" s="7"/>
     </row>
@@ -1294,22 +1327,22 @@
         <v>7</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>52</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>79</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J16" s="9">
         <v>3</v>
@@ -1326,25 +1359,25 @@
         <v>7</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J17" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K17" s="7"/>
     </row>
@@ -1355,62 +1388,126 @@
         <v>16</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="J18" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
       </c>
       <c r="K19" s="7"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1"/>
+      <c r="B20" s="11">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" s="9">
+        <v>1</v>
+      </c>
+      <c r="K20" s="9"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1"/>
+      <c r="B21" s="11">
+        <f>ROW(B21) - ROW($B$2)</f>
+        <v>19</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="I21" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="J21" s="7">
+        <v>1</v>
+      </c>
+      <c r="K21" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>